<commit_message>
Added link to PDF slides. Added meetup.
</commit_message>
<xml_diff>
--- a/Schedule.xlsx
+++ b/Schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Dropbox/SPS Dropbox/Jason Bryer/Teaching/IS381 2026 Spring/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74A7B0B3-C5FE-C141-B9F1-5A963DBA8B9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17B70F6E-3B4B-C349-9A30-190608D9C722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5000" yWindow="11820" windowWidth="24780" windowHeight="14160" xr2:uid="{BFE2A6F7-E8E8-014E-9460-2468D969C60C}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>Week</t>
   </si>
@@ -225,6 +225,12 @@
   </si>
   <si>
     <t>wIJV74NhoRU</t>
+  </si>
+  <si>
+    <t>07-Distributions</t>
+  </si>
+  <si>
+    <t>GGLXCtG0fn0</t>
   </si>
 </sst>
 </file>
@@ -1360,6 +1366,12 @@
       <c r="G8" t="s">
         <v>23</v>
       </c>
+      <c r="H8" t="s">
+        <v>64</v>
+      </c>
+      <c r="I8" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="2">

</xml_diff>